<commit_message>
Change unit to uom and average to regular
</commit_message>
<xml_diff>
--- a/public/templates/template-pm-request.xlsx
+++ b/public/templates/template-pm-request.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marth\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28AB329F-6627-4CD2-BA85-916BF956A06A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47746C16-EC98-45F0-8E6E-DD59CC97AB81}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{206DC4D3-AD0A-4DF7-B945-16D682D170FD}"/>
   </bookViews>
@@ -46,9 +46,6 @@
     <t>Item</t>
   </si>
   <si>
-    <t>Unit</t>
-  </si>
-  <si>
     <t>Qty</t>
   </si>
   <si>
@@ -89,6 +86,9 @@
   </si>
   <si>
     <t>Price</t>
+  </si>
+  <si>
+    <t>Uom</t>
   </si>
 </sst>
 </file>
@@ -504,7 +504,7 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="3" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.3">
@@ -515,22 +515,22 @@
         <v>2</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D3" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E3" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="E3" s="5" t="s">
+      <c r="F3" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="F3" s="6" t="s">
-        <v>5</v>
-      </c>
       <c r="G3" s="5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H3" s="8" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.3">
@@ -538,13 +538,13 @@
         <v>1</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E4" s="3">
         <v>2</v>
@@ -553,7 +553,7 @@
         <v>45912</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H4" s="9">
         <v>200000</v>
@@ -564,13 +564,13 @@
         <v>2</v>
       </c>
       <c r="B5" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C5" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="D5" s="3" t="s">
         <v>15</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>16</v>
       </c>
       <c r="E5" s="3">
         <v>50</v>
@@ -579,7 +579,7 @@
         <v>45789</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="H5" s="9">
         <v>78600</v>
@@ -590,13 +590,13 @@
         <v>3</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E6" s="3">
         <v>2</v>
@@ -605,7 +605,7 @@
         <v>45912</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H6" s="9">
         <v>425000</v>
@@ -616,13 +616,13 @@
         <v>4</v>
       </c>
       <c r="B7" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C7" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="D7" s="3" t="s">
         <v>15</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>16</v>
       </c>
       <c r="E7" s="3">
         <v>50</v>
@@ -631,7 +631,7 @@
         <v>45789</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="H7" s="9">
         <v>21000</v>
@@ -1096,17 +1096,17 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>